<commit_message>
Quelques corrections dans l'activité excel.
</commit_message>
<xml_diff>
--- a/docs/2e/bases-de-donnees/meteo-corrige.xlsx
+++ b/docs/2e/bases-de-donnees/meteo-corrige.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caro\Documents\Projets\t-doc\informatique\docs\2e\bases-de-donnees\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5AF5C48-AD42-44E2-9010-BB22000476B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A50765E-A1E6-48FC-9810-F2C8B8056ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11760" xr2:uid="{E8FB6D54-8182-47F2-A6BF-6FB10867FC41}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="23">
   <si>
     <t>Jan</t>
   </si>
@@ -92,9 +92,6 @@
     <t>Dec</t>
   </si>
   <si>
-    <t>Geneve</t>
-  </si>
-  <si>
     <t>Températures minimales moyennes (en °C)</t>
   </si>
   <si>
@@ -102,6 +99,12 @@
   </si>
   <si>
     <t>Moyenne</t>
+  </si>
+  <si>
+    <t>Genève</t>
+  </si>
+  <si>
+    <t>M &gt; M Suiss</t>
   </si>
 </sst>
 </file>
@@ -158,7 +161,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -186,125 +189,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
         </patternFill>
       </fill>
     </dxf>
@@ -391,7 +275,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="fr-CH"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -828,7 +712,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="fr-CH"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1888,6 +1772,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1494924528"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -3604,16 +3489,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>288925</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>288925</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>146050</xdr:rowOff>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3640,16 +3525,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>330200</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>44450</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>330200</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>44450</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4030,15 +3915,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30FEB678-26B2-49A4-9AF7-15B31462EF99}">
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.90625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -4053,7 +3938,7 @@
       <c r="L1" s="3"/>
       <c r="M1" s="3"/>
     </row>
-    <row r="2" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
       <c r="B2" s="1" t="s">
         <v>0</v>
@@ -4092,10 +3977,13 @@
         <v>17</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -4139,8 +4027,12 @@
         <f>ROUND(AVERAGE(B3:M3),1)</f>
         <v>4.8</v>
       </c>
+      <c r="O3" t="str">
+        <f>IF(N3&gt;$N$9,"OUI","NON")</f>
+        <v>NON</v>
+      </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -4181,13 +4073,17 @@
         <v>-3.3</v>
       </c>
       <c r="N4">
-        <f t="shared" ref="N4:N8" si="0">ROUND(AVERAGE(B4:M4),1)</f>
+        <f t="shared" ref="N4:N9" si="0">ROUND(AVERAGE(B4:M4),1)</f>
         <v>3.5</v>
       </c>
+      <c r="O4" t="str">
+        <f t="shared" ref="O4:O8" si="1">IF(N4&gt;$N$9,"OUI","NON")</f>
+        <v>NON</v>
+      </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B5">
         <v>-2</v>
@@ -4229,8 +4125,12 @@
         <f t="shared" si="0"/>
         <v>5.9</v>
       </c>
+      <c r="O5" t="str">
+        <f t="shared" si="1"/>
+        <v>OUI</v>
+      </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -4274,8 +4174,12 @@
         <f t="shared" si="0"/>
         <v>8.1</v>
       </c>
+      <c r="O6" t="str">
+        <f t="shared" si="1"/>
+        <v>OUI</v>
+      </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
@@ -4319,8 +4223,12 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
+      <c r="O7" t="str">
+        <f t="shared" si="1"/>
+        <v>OUI</v>
+      </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
@@ -4364,63 +4272,71 @@
         <f t="shared" si="0"/>
         <v>5.8</v>
       </c>
+      <c r="O8" t="str">
+        <f t="shared" si="1"/>
+        <v>OUI</v>
+      </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9">
         <f>ROUND(AVERAGE(B3:B8),1)</f>
         <v>-2.2999999999999998</v>
       </c>
       <c r="C9">
-        <f t="shared" ref="C9:M9" si="1">ROUND(AVERAGE(C3:C8),1)</f>
+        <f t="shared" ref="C9:M9" si="2">ROUND(AVERAGE(C3:C8),1)</f>
         <v>-2.1</v>
       </c>
       <c r="D9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.7</v>
       </c>
       <c r="E9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.0999999999999996</v>
       </c>
       <c r="F9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="G9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>12.2</v>
       </c>
       <c r="H9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14.4</v>
       </c>
       <c r="I9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14.3</v>
       </c>
       <c r="J9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>10.9</v>
       </c>
       <c r="K9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.1</v>
       </c>
       <c r="L9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.2000000000000002</v>
       </c>
       <c r="M9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1.2</v>
       </c>
+      <c r="N9">
+        <f t="shared" si="0"/>
+        <v>5.7</v>
+      </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -4435,7 +4351,7 @@
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
     </row>
-    <row r="12" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>0</v>
       </c>
@@ -4472,8 +4388,11 @@
       <c r="M12" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="O12" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>5</v>
       </c>
@@ -4517,8 +4436,12 @@
         <f>ROUND(AVERAGE(B13:M13),1)</f>
         <v>12.9</v>
       </c>
+      <c r="O13" t="str">
+        <f>IF(N13&gt;$N$19,"OUI","NON")</f>
+        <v>NON</v>
+      </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>8</v>
       </c>
@@ -4559,13 +4482,17 @@
         <v>3.6</v>
       </c>
       <c r="N14">
-        <f t="shared" ref="N14:N18" si="2">ROUND(AVERAGE(B14:M14),1)</f>
+        <f t="shared" ref="N14:N19" si="3">ROUND(AVERAGE(B14:M14),1)</f>
         <v>12.2</v>
       </c>
+      <c r="O14" t="str">
+        <f t="shared" ref="O14:O18" si="4">IF(N14&gt;$N$19,"OUI","NON")</f>
+        <v>NON</v>
+      </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B15">
         <v>4</v>
@@ -4604,11 +4531,15 @@
         <v>5</v>
       </c>
       <c r="N15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>13.9</v>
       </c>
+      <c r="O15" t="str">
+        <f t="shared" si="4"/>
+        <v>OUI</v>
+      </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>6</v>
       </c>
@@ -4649,11 +4580,15 @@
         <v>6</v>
       </c>
       <c r="N16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
+      <c r="O16" t="str">
+        <f t="shared" si="4"/>
+        <v>OUI</v>
+      </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
@@ -4694,11 +4629,15 @@
         <v>4.8</v>
       </c>
       <c r="N17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>13.6</v>
       </c>
+      <c r="O17" t="str">
+        <f t="shared" si="4"/>
+        <v>OUI</v>
+      </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>4</v>
       </c>
@@ -4739,64 +4678,72 @@
         <v>4.9000000000000004</v>
       </c>
       <c r="N18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>13.8</v>
       </c>
+      <c r="O18" t="str">
+        <f t="shared" si="4"/>
+        <v>OUI</v>
+      </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19">
         <f>ROUND(AVERAGE(B13:B18),1)</f>
         <v>3.8</v>
       </c>
       <c r="C19">
-        <f t="shared" ref="C19:M19" si="3">ROUND(AVERAGE(C13:C18),1)</f>
+        <f t="shared" ref="C19:M19" si="5">ROUND(AVERAGE(C13:C18),1)</f>
         <v>5</v>
       </c>
       <c r="D19">
+        <f t="shared" si="5"/>
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="5"/>
+        <v>13.3</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="5"/>
+        <v>17</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="5"/>
+        <v>21.1</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="5"/>
+        <v>22.9</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="5"/>
+        <v>22.6</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="5"/>
+        <v>18.5</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="5"/>
+        <v>14.3</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="5"/>
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="5"/>
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="N19">
         <f t="shared" si="3"/>
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="E19">
-        <f t="shared" si="3"/>
-        <v>13.3</v>
-      </c>
-      <c r="F19">
-        <f t="shared" si="3"/>
-        <v>17</v>
-      </c>
-      <c r="G19">
-        <f t="shared" si="3"/>
-        <v>21.1</v>
-      </c>
-      <c r="H19">
-        <f t="shared" si="3"/>
-        <v>22.9</v>
-      </c>
-      <c r="I19">
-        <f t="shared" si="3"/>
-        <v>22.6</v>
-      </c>
-      <c r="J19">
-        <f t="shared" si="3"/>
-        <v>18.5</v>
-      </c>
-      <c r="K19">
-        <f t="shared" si="3"/>
-        <v>14.3</v>
-      </c>
-      <c r="L19">
-        <f t="shared" si="3"/>
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="M19">
-        <f t="shared" si="3"/>
-        <v>4.5999999999999996</v>
+        <v>13.4</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>9</v>
       </c>
@@ -4813,7 +4760,7 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>
-    <row r="22" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B22" s="1" t="s">
         <v>0</v>
       </c>
@@ -4851,7 +4798,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>5</v>
       </c>
@@ -4896,7 +4843,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>8</v>
       </c>
@@ -4937,13 +4884,13 @@
         <v>122</v>
       </c>
       <c r="N24">
-        <f t="shared" ref="N24:N28" si="4">SUM(B24:M24)</f>
+        <f t="shared" ref="N24:N28" si="6">SUM(B24:M24)</f>
         <v>1530</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B25">
         <v>118</v>
@@ -4982,11 +4929,11 @@
         <v>133</v>
       </c>
       <c r="N25">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1468</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>6</v>
       </c>
@@ -5027,11 +4974,11 @@
         <v>128</v>
       </c>
       <c r="N26">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1350</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>7</v>
       </c>
@@ -5072,11 +5019,11 @@
         <v>80</v>
       </c>
       <c r="N27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1658</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>4</v>
       </c>
@@ -5117,13 +5064,13 @@
         <v>111</v>
       </c>
       <c r="N28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1463</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N29">
         <f>ROUND(AVERAGE(N23:N28), 0)</f>
@@ -5140,6 +5087,18 @@
     <mergeCell ref="A21:M21"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:M8">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B13:M18">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -5151,20 +5110,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B13:M18">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B23:M28">
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -5174,7 +5121,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N23:N28">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+      <formula>$N$29</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <formula>$N$29</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>